<commit_message>
Stabilise demo workflows and helper guardrails
</commit_message>
<xml_diff>
--- a/dataset/DevelopmentBenchmark/Task04/final_schedule.xlsx
+++ b/dataset/DevelopmentBenchmark/Task04/final_schedule.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final Schedule" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Final Schedule" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Data Cleanup</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
     </row>
@@ -478,22 +478,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Feature Extraction</t>
+          <t>Data Ingestion</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>10:30</t>
         </is>
       </c>
     </row>
@@ -505,22 +505,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Model Training</t>
+          <t>Data Cleaning</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>11:30</t>
         </is>
       </c>
     </row>
@@ -532,22 +532,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Report Generation</t>
+          <t>Feature Engineering</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>13:30</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Validation Checks</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -569,12 +569,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>14:30</t>
         </is>
       </c>
     </row>
@@ -586,33 +586,143 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Export Results</t>
+          <t>Model Training</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Compliance Review</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>21:00</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>22:00</t>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Evaluation Report</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>19:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Client Pack</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Final Export</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Total Duration (hours)</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>14</v>
+      <c r="B14" t="n">
+        <v>13.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>